<commit_message>
Package 18 validation update
</commit_message>
<xml_diff>
--- a/curation/draft/package18/R18_BC_DSS_BrCa_TAUG.xlsx
+++ b/curation/draft/package18/R18_BC_DSS_BrCa_TAUG.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_github\cdisc-org\COSMoS\curation\draft\package18\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F3BCA83-3D65-484B-B269-B299B23C8A73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50D212C5-0B53-449C-B5DF-5690C9990982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{9C2B54C0-060B-496F-B408-7D0F2041239C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{9C2B54C0-060B-496F-B408-7D0F2041239C}"/>
   </bookViews>
   <sheets>
     <sheet name="BC_BrCa" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4220" uniqueCount="521">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4216" uniqueCount="522">
   <si>
     <t>package_date</t>
   </si>
@@ -1607,6 +1607,9 @@
   </si>
   <si>
     <t>NEW_DEC2</t>
+  </si>
+  <si>
+    <t>QRS;Clinical or Research Assessment Classification;AJCC Cancer Staging Manual</t>
   </si>
 </sst>
 </file>
@@ -4045,7 +4048,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:17" ht="39" x14ac:dyDescent="0.25">
       <c r="A42" s="7" t="s">
         <v>58</v>
       </c>
@@ -4061,7 +4064,9 @@
       <c r="E42" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="F42" s="5"/>
+      <c r="F42" s="5" t="s">
+        <v>521</v>
+      </c>
       <c r="G42" s="4" t="s">
         <v>222</v>
       </c>
@@ -14042,9 +14047,7 @@
       </c>
       <c r="AC93" s="4"/>
       <c r="AD93" s="4"/>
-      <c r="AE93" s="4" t="s">
-        <v>169</v>
-      </c>
+      <c r="AE93" s="4"/>
       <c r="AF93" s="4"/>
     </row>
     <row r="94" spans="1:32" x14ac:dyDescent="0.25">
@@ -14594,9 +14597,7 @@
       </c>
       <c r="AC100" s="4"/>
       <c r="AD100" s="4"/>
-      <c r="AE100" s="4" t="s">
-        <v>169</v>
-      </c>
+      <c r="AE100" s="4"/>
       <c r="AF100" s="4"/>
     </row>
     <row r="101" spans="1:32" x14ac:dyDescent="0.25">
@@ -15146,9 +15147,7 @@
       </c>
       <c r="AC107" s="4"/>
       <c r="AD107" s="4"/>
-      <c r="AE107" s="4" t="s">
-        <v>169</v>
-      </c>
+      <c r="AE107" s="4"/>
       <c r="AF107" s="4"/>
     </row>
     <row r="108" spans="1:32" x14ac:dyDescent="0.25">
@@ -15698,9 +15697,7 @@
       </c>
       <c r="AC114" s="4"/>
       <c r="AD114" s="4"/>
-      <c r="AE114" s="4" t="s">
-        <v>169</v>
-      </c>
+      <c r="AE114" s="4"/>
       <c r="AF114" s="4"/>
     </row>
     <row r="115" spans="1:32" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -16250,9 +16247,7 @@
       </c>
       <c r="AC121" s="4"/>
       <c r="AD121" s="4"/>
-      <c r="AE121" s="4" t="s">
-        <v>169</v>
-      </c>
+      <c r="AE121" s="4"/>
       <c r="AF121" s="4"/>
     </row>
     <row r="122" spans="1:32" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>